<commit_message>
Stage 8 review fixes: D-012
</commit_message>
<xml_diff>
--- a/output/archive/QuenverellData/engagements/qv.25.103/docking/procurement/dt8-ranked-hitlist-DRAFT-v2.xlsx
+++ b/output/archive/QuenverellData/engagements/qv.25.103/docking/procurement/dt8-ranked-hitlist-DRAFT-v2.xlsx
@@ -153,9 +153,9 @@
     <author>Nadia Rahmani</author>
   </authors>
   <commentList>
-    <comment ref="E4" authorId="0" shapeId="0">
+    <comment ref="E2" authorId="0" shapeId="0">
       <text>
-        <t>Series 2 scaffold ownership not settled. Do not order until Drelvessa confirms.</t>
+        <t>Scaffold ownership remains unresolved. Consult client chemistry correspondence; do not order.</t>
       </text>
     </comment>
   </commentList>
@@ -649,7 +649,7 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Ligand</t>
+          <t>Ligand source record</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
@@ -659,12 +659,12 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Second protonation set</t>
+          <t>Preparation record</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Scaffold</t>
+          <t>Scaffold review</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
@@ -674,12 +674,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="A2" s="3" t="inlineStr"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Ligand A</t>
+          <t>Engagement ranked hit list</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -694,76 +692,34 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Series 1</t>
+          <t>[TBC]</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Ranked, pending scaffold check</t>
+          <t>Draft; procurement on hold</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Ligand B</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>[TBC]</t>
-        </is>
-      </c>
+      <c r="A3" s="3" t="inlineStr"/>
+      <c r="B3" s="3" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Series 1</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Ranked, pending scaffold check</t>
-        </is>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Ligand C</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>[TBC]</t>
-        </is>
-      </c>
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr"/>
       <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Series 2</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Under review</t>
-        </is>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Ligand D</t>
-        </is>
-      </c>
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr"/>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
@@ -845,7 +801,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Which Drelvessa team owns the Series 2 scaffold, and whether it can be sourced for DT-8</t>
+          <t>Scaffold ownership question remains with the Drelvessa chemistry team; resolution [TBC].</t>
         </is>
       </c>
     </row>
@@ -901,7 +857,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Re-rank once the scaffold question is answered; the Ranked list sheet is not final</t>
+          <t>Await the client ownership decision before completing procurement review; retain the draft ranking in the engagement records.</t>
         </is>
       </c>
     </row>

</xml_diff>